<commit_message>
fix(bi-indices): preserva unicidade de provisorios PR com RECNO e corrige totais (v8.99)
</commit_message>
<xml_diff>
--- a/14-CONTAS-A-PAGAR-2026-08-31.xlsx
+++ b/14-CONTAS-A-PAGAR-2026-08-31.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexandre\Documents\Gemini-Cli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09624115-781E-4223-8B38-5B44D677463D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607D9A95-8CF2-44AD-9667-815AF4BD1596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1A064813-1C56-48D5-B186-72776F96DCD4}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1231" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="126">
   <si>
     <t>Dt.Ref: 31/08/2026</t>
   </si>
@@ -411,16 +411,13 @@
   </si>
   <si>
     <t>AE</t>
-  </si>
-  <si>
-    <t>SEM PA:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="8"/>
       <name val="Courier New"/>
@@ -535,11 +532,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Courier New"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="33">
@@ -892,19 +884,19 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -913,10 +905,7 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1303,7 +1292,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E4F7969-50EB-46F7-87BC-232B2912664C}">
-  <dimension ref="A1:AJ53"/>
+  <dimension ref="A1:AJ57"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -1478,7 +1467,7 @@
       <c r="E5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="6">
         <v>1900</v>
       </c>
       <c r="G5" s="2">
@@ -1588,7 +1577,7 @@
       <c r="E6" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="6">
         <v>5318.72</v>
       </c>
       <c r="G6" s="2">
@@ -1698,7 +1687,7 @@
       <c r="E7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="6">
         <v>7571.32</v>
       </c>
       <c r="G7" s="2">
@@ -1808,7 +1797,7 @@
       <c r="E8" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="6">
         <v>604.92999999999995</v>
       </c>
       <c r="G8" s="2">
@@ -1918,7 +1907,7 @@
       <c r="E9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="6">
         <v>772.31</v>
       </c>
       <c r="G9" s="2">
@@ -2028,7 +2017,7 @@
       <c r="E10" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="6">
         <v>393.1</v>
       </c>
       <c r="G10" s="2">
@@ -2248,7 +2237,7 @@
       <c r="E12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="6">
         <v>1460.37</v>
       </c>
       <c r="G12" s="2">
@@ -2358,7 +2347,7 @@
       <c r="E13" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="6">
         <v>546.89</v>
       </c>
       <c r="G13" s="2">
@@ -2468,7 +2457,7 @@
       <c r="E14" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="6">
         <v>235.74</v>
       </c>
       <c r="G14" s="2">
@@ -2578,7 +2567,7 @@
       <c r="E15" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="6">
         <v>774</v>
       </c>
       <c r="G15" s="2">
@@ -2688,7 +2677,7 @@
       <c r="E16" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="6">
         <v>1336.4</v>
       </c>
       <c r="G16" s="2">
@@ -2798,7 +2787,7 @@
       <c r="E17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="6">
         <v>3356.14</v>
       </c>
       <c r="G17" s="2">
@@ -3018,7 +3007,7 @@
       <c r="E19" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="6">
         <v>5318.72</v>
       </c>
       <c r="G19" s="2">
@@ -3128,7 +3117,7 @@
       <c r="E20" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="6">
         <v>526.54999999999995</v>
       </c>
       <c r="G20" s="2">
@@ -3238,7 +3227,7 @@
       <c r="E21" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="6">
         <v>393.1</v>
       </c>
       <c r="G21" s="2">
@@ -3348,7 +3337,7 @@
       <c r="E22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="6">
         <v>772.31</v>
       </c>
       <c r="G22" s="2">
@@ -3458,7 +3447,7 @@
       <c r="E23" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="6">
         <v>15000</v>
       </c>
       <c r="G23" s="2">
@@ -3568,7 +3557,7 @@
       <c r="E24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="6">
         <v>1460.37</v>
       </c>
       <c r="G24" s="2">
@@ -3788,7 +3777,7 @@
       <c r="E26" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="6">
         <v>4579.34</v>
       </c>
       <c r="G26" s="2">
@@ -3898,7 +3887,7 @@
       <c r="E27" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="6">
         <v>5100</v>
       </c>
       <c r="G27" s="2">
@@ -4008,7 +3997,7 @@
       <c r="E28" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="6">
         <v>350</v>
       </c>
       <c r="G28" s="2">
@@ -4118,7 +4107,7 @@
       <c r="E29" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="6">
         <v>772.31</v>
       </c>
       <c r="G29" s="2">
@@ -4228,7 +4217,7 @@
       <c r="E30" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="6">
         <v>1460.37</v>
       </c>
       <c r="G30" s="2">
@@ -4338,7 +4327,7 @@
       <c r="E31" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F31" s="6">
         <v>4579.34</v>
       </c>
       <c r="G31" s="2">
@@ -4558,7 +4547,7 @@
       <c r="E33" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="6">
         <v>59</v>
       </c>
       <c r="G33" s="2">
@@ -4668,7 +4657,7 @@
       <c r="E34" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="6">
         <v>5318.71</v>
       </c>
       <c r="G34" s="2">
@@ -4778,7 +4767,7 @@
       <c r="E35" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="F35" s="8">
+      <c r="F35" s="6">
         <v>20000</v>
       </c>
       <c r="G35" s="2">
@@ -4888,7 +4877,7 @@
       <c r="E36" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="6">
         <v>604.91999999999996</v>
       </c>
       <c r="G36" s="2">
@@ -4998,7 +4987,7 @@
       <c r="E37" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="6">
         <v>417.9</v>
       </c>
       <c r="G37" s="2">
@@ -5108,7 +5097,7 @@
       <c r="E38" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="6">
         <v>393.1</v>
       </c>
       <c r="G38" s="2">
@@ -5328,7 +5317,7 @@
       <c r="E40" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F40" s="6">
         <v>245</v>
       </c>
       <c r="G40" s="2">
@@ -5438,7 +5427,7 @@
       <c r="E41" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F41" s="8">
+      <c r="F41" s="6">
         <v>1460.37</v>
       </c>
       <c r="G41" s="2">
@@ -5548,7 +5537,7 @@
       <c r="E42" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F42" s="6">
         <v>4579.34</v>
       </c>
       <c r="G42" s="2">
@@ -5658,7 +5647,7 @@
       <c r="E43" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="F43" s="8">
+      <c r="F43" s="6">
         <v>400</v>
       </c>
       <c r="G43" s="2">
@@ -5768,7 +5757,7 @@
       <c r="E44" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="F44" s="8">
+      <c r="F44" s="6">
         <v>2502.75</v>
       </c>
       <c r="G44" s="2">
@@ -5878,7 +5867,7 @@
       <c r="E45" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F45" s="8">
+      <c r="F45" s="6">
         <v>772.31</v>
       </c>
       <c r="G45" s="2">
@@ -6098,7 +6087,7 @@
       <c r="E47" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F47" s="8">
+      <c r="F47" s="6">
         <v>4579.34</v>
       </c>
       <c r="G47" s="2">
@@ -6208,7 +6197,7 @@
       <c r="E48" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F48" s="8">
+      <c r="F48" s="6">
         <v>1460.36</v>
       </c>
       <c r="G48" s="2">
@@ -6318,7 +6307,7 @@
       <c r="E49" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F49" s="8">
+      <c r="F49" s="6">
         <v>4579.3599999999997</v>
       </c>
       <c r="G49" s="2">
@@ -6412,23 +6401,61 @@
         <v>43</v>
       </c>
     </row>
+    <row r="51" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A51" s="6"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6"/>
+      <c r="E51" s="6"/>
+    </row>
     <row r="52" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="F52" s="6">
-        <f>SUM(F5:F49)</f>
+      <c r="A52" s="6"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6"/>
+      <c r="Q52" s="8">
+        <f>SUM(Q5:Q49)</f>
         <v>111954.79000000001</v>
       </c>
     </row>
     <row r="53" spans="1:36" x14ac:dyDescent="0.2">
-      <c r="E53" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="F53" s="6">
-        <f>F52</f>
-        <v>111954.79000000001</v>
-      </c>
+      <c r="A53" s="6"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+    </row>
+    <row r="54" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A54" s="6"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+    </row>
+    <row r="55" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A55" s="6"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+    </row>
+    <row r="56" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
+    </row>
+    <row r="57" spans="1:36" x14ac:dyDescent="0.2">
+      <c r="A57" s="6"/>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="6"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:D1048576">
+  <conditionalFormatting sqref="D1:D50 D58:D1048576">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"PA"</formula>
     </cfRule>

</xml_diff>